<commit_message>
Add BESS bankability blog article, RFI system, warranties docs, and group proposal updates
- New blog: BESS Bankability — why choosing the right service partner matters,
  covering Linyang-Lighthief OEM partnership, multi-layered insurance structure,
  and lender bankability requirements
- Add blog card to listing page as featured article
- Add RFI API routes and service layer with Supabase migration
- Add BESS procurement page
- Add warranties and insurance documentation (MD + HTML)
- Update all 6 group proposals with expanded content
- Update EPC readiness assessment, scope pricing tracker, and pricing verification
- Update EPC system cost spreadsheet

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Bess - EPC System Cost v2.xlsx
+++ b/docs/Bess - EPC System Cost v2.xlsx
@@ -19,7 +19,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="€#,##0.00"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -121,6 +121,15 @@
     <font>
       <b val="1"/>
       <color rgb="00FF0000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
     </font>
   </fonts>
   <fills count="35">
@@ -361,7 +370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -691,6 +700,15 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1576,7 +1594,7 @@
           <t>Docs &amp; Statutory Compliance (EAC / CERA fees only) Estimate 7000</t>
         </is>
       </c>
-      <c r="AN2" s="16" t="n">
+      <c r="AN2" s="160" t="n">
         <v>0.0075</v>
       </c>
       <c r="AO2" s="17" t="n"/>
@@ -1698,9 +1716,9 @@
           <t>Confirmed from Dino this is on Clieent\</t>
         </is>
       </c>
-      <c r="AN3" s="107" t="inlineStr">
-        <is>
-          <t>Need qoute. double check if RFP is properly allocating all needs</t>
+      <c r="AN3" s="161" t="inlineStr">
+        <is>
+          <t>✅ VERIFIED — Agent confirmed 0.75% of CIF. Feb 2026.</t>
         </is>
       </c>
       <c r="AO3" s="107" t="inlineStr">
@@ -1846,7 +1864,10 @@
       <c r="AK4" s="130" t="n"/>
       <c r="AL4" s="130" t="n"/>
       <c r="AM4" s="130" t="n"/>
-      <c r="AN4" s="130" t="n"/>
+      <c r="AN4" s="36">
+        <f>Q4*$AN$2</f>
+        <v/>
+      </c>
       <c r="AO4" s="130" t="n"/>
       <c r="AP4" s="130">
         <f>SUM(T4,U4,V4,W4,X4,Y4,Z4,AA4,AB4,AC4,AD4,AE4,AF4,AG4,AH4,AJ4,AK4,AL4,AM4,AN4,AO4)</f>
@@ -2077,8 +2098,8 @@
         <v>0</v>
       </c>
       <c r="AM5" s="130" t="n"/>
-      <c r="AN5" s="130">
-        <f>N11*0.0075</f>
+      <c r="AN5" s="36">
+        <f>Q5*$AN$2</f>
         <v/>
       </c>
       <c r="AO5" s="130" t="n">
@@ -2314,8 +2335,8 @@
         <v>0</v>
       </c>
       <c r="AM6" s="131" t="n"/>
-      <c r="AN6" s="135">
-        <f>N12*0.0075</f>
+      <c r="AN6" s="162">
+        <f>Q6*$AN$2</f>
         <v/>
       </c>
       <c r="AO6" s="135" t="n">
@@ -2525,7 +2546,10 @@
       <c r="AK7" s="130" t="n"/>
       <c r="AL7" s="130" t="n"/>
       <c r="AM7" s="130" t="n"/>
-      <c r="AN7" s="130" t="n"/>
+      <c r="AN7" s="36">
+        <f>Q7*$AN$2</f>
+        <v/>
+      </c>
       <c r="AO7" s="130" t="n"/>
       <c r="AP7" s="130">
         <f>SUM(T7,U7,V7,W7,X7,Y7,Z7,AA7,AB7,AC7,AD7,AE7,AF7,AG7,AH7,AJ7,AK7,AL7,AM7,AN7,AO7)</f>
@@ -2756,8 +2780,8 @@
         <v>0</v>
       </c>
       <c r="AM8" s="130" t="n"/>
-      <c r="AN8" s="130">
-        <f>N25*0.0075</f>
+      <c r="AN8" s="36">
+        <f>Q8*$AN$2</f>
         <v/>
       </c>
       <c r="AO8" s="130" t="n">
@@ -2993,8 +3017,8 @@
         <v>0</v>
       </c>
       <c r="AM9" s="130" t="n"/>
-      <c r="AN9" s="130">
-        <f>N31*0.0075</f>
+      <c r="AN9" s="36">
+        <f>Q9*$AN$2</f>
         <v/>
       </c>
       <c r="AO9" s="130" t="n">
@@ -3230,8 +3254,8 @@
         <v>0</v>
       </c>
       <c r="AM10" s="130" t="n"/>
-      <c r="AN10" s="130">
-        <f>N32*0.0075</f>
+      <c r="AN10" s="36">
+        <f>Q10*$AN$2</f>
         <v/>
       </c>
       <c r="AO10" s="130" t="n">
@@ -3469,8 +3493,8 @@
         <v>0</v>
       </c>
       <c r="AM11" s="130" t="n"/>
-      <c r="AN11" s="130">
-        <f>N37*0.0075</f>
+      <c r="AN11" s="36">
+        <f>Q11*$AN$2</f>
         <v/>
       </c>
       <c r="AO11" s="130" t="n">
@@ -3708,8 +3732,8 @@
         <v>0</v>
       </c>
       <c r="AM12" s="131" t="n"/>
-      <c r="AN12" s="135">
-        <f>N38*0.0075</f>
+      <c r="AN12" s="162">
+        <f>Q12*$AN$2</f>
         <v/>
       </c>
       <c r="AO12" s="135" t="n">
@@ -3947,8 +3971,8 @@
         <v>0</v>
       </c>
       <c r="AM13" s="130" t="n"/>
-      <c r="AN13" s="130">
-        <f>N39*0.0075</f>
+      <c r="AN13" s="36">
+        <f>Q13*$AN$2</f>
         <v/>
       </c>
       <c r="AO13" s="130" t="n">
@@ -4186,8 +4210,8 @@
         <v>0</v>
       </c>
       <c r="AM14" s="130" t="n"/>
-      <c r="AN14" s="130">
-        <f>N40*0.0075</f>
+      <c r="AN14" s="36">
+        <f>Q14*$AN$2</f>
         <v/>
       </c>
       <c r="AO14" s="130" t="n">
@@ -4425,8 +4449,8 @@
         <v>0</v>
       </c>
       <c r="AM15" s="130" t="n"/>
-      <c r="AN15" s="130">
-        <f>N41*0.0075</f>
+      <c r="AN15" s="36">
+        <f>Q15*$AN$2</f>
         <v/>
       </c>
       <c r="AO15" s="130" t="n">
@@ -4662,8 +4686,8 @@
         <v>0</v>
       </c>
       <c r="AM16" s="130" t="n"/>
-      <c r="AN16" s="130">
-        <f>N23*0.0075</f>
+      <c r="AN16" s="36">
+        <f>Q16*$AN$2</f>
         <v/>
       </c>
       <c r="AO16" s="130" t="n">
@@ -4897,8 +4921,8 @@
         <v>0</v>
       </c>
       <c r="AM17" s="130" t="n"/>
-      <c r="AN17" s="130">
-        <f>N24*0.0075</f>
+      <c r="AN17" s="36">
+        <f>Q17*$AN$2</f>
         <v/>
       </c>
       <c r="AO17" s="130" t="n">
@@ -5132,8 +5156,8 @@
         <v>0</v>
       </c>
       <c r="AM18" s="130" t="n"/>
-      <c r="AN18" s="130">
-        <f>N28*0.0075</f>
+      <c r="AN18" s="36">
+        <f>Q18*$AN$2</f>
         <v/>
       </c>
       <c r="AO18" s="130" t="n">
@@ -5367,8 +5391,8 @@
         <v>0</v>
       </c>
       <c r="AM19" s="130" t="n"/>
-      <c r="AN19" s="130">
-        <f>N29*0.0075</f>
+      <c r="AN19" s="36">
+        <f>Q19*$AN$2</f>
         <v/>
       </c>
       <c r="AO19" s="130" t="n">
@@ -5602,8 +5626,8 @@
         <v>0</v>
       </c>
       <c r="AM20" s="130" t="n"/>
-      <c r="AN20" s="130">
-        <f>N27*0.0075</f>
+      <c r="AN20" s="36">
+        <f>Q20*$AN$2</f>
         <v/>
       </c>
       <c r="AO20" s="130" t="n">
@@ -5837,8 +5861,8 @@
         <v>0</v>
       </c>
       <c r="AM21" s="130" t="n"/>
-      <c r="AN21" s="130">
-        <f>N33*0.0075</f>
+      <c r="AN21" s="36">
+        <f>Q21*$AN$2</f>
         <v/>
       </c>
       <c r="AO21" s="130" t="n">
@@ -6072,8 +6096,8 @@
         <v>0</v>
       </c>
       <c r="AM22" s="130" t="n"/>
-      <c r="AN22" s="130">
-        <f>N34*0.0075</f>
+      <c r="AN22" s="36">
+        <f>Q22*$AN$2</f>
         <v/>
       </c>
       <c r="AO22" s="130" t="n">
@@ -6307,8 +6331,8 @@
         <v>0</v>
       </c>
       <c r="AM23" s="130" t="n"/>
-      <c r="AN23" s="130">
-        <f>N35*0.0075</f>
+      <c r="AN23" s="36">
+        <f>Q23*$AN$2</f>
         <v/>
       </c>
       <c r="AO23" s="130" t="n">
@@ -6544,8 +6568,8 @@
         <v>0</v>
       </c>
       <c r="AM24" s="130" t="n"/>
-      <c r="AN24" s="130">
-        <f>N30*0.0075</f>
+      <c r="AN24" s="36">
+        <f>Q24*$AN$2</f>
         <v/>
       </c>
       <c r="AO24" s="130" t="n">
@@ -6750,7 +6774,10 @@
       <c r="AK25" s="131" t="n"/>
       <c r="AL25" s="131" t="n"/>
       <c r="AM25" s="131" t="n"/>
-      <c r="AN25" s="131" t="n"/>
+      <c r="AN25" s="78">
+        <f>Q25*$AN$2</f>
+        <v/>
+      </c>
       <c r="AO25" s="131" t="n"/>
       <c r="AP25" s="135">
         <f>SUM(T25,U25,V25,W25,X25,Y25,Z25,AA25,AB25,AC25,AD25,AE25,AF25,AG25,AH25,AJ25,AK25,AL25,AM25,AN25,AO25)</f>
@@ -6983,8 +7010,8 @@
         <v>0</v>
       </c>
       <c r="AM26" s="130" t="n"/>
-      <c r="AN26" s="130">
-        <f>N36*0.0075</f>
+      <c r="AN26" s="36">
+        <f>Q26*$AN$2</f>
         <v/>
       </c>
       <c r="AO26" s="130" t="n">
@@ -7191,7 +7218,10 @@
       <c r="AK27" s="131" t="n"/>
       <c r="AL27" s="131" t="n"/>
       <c r="AM27" s="131" t="n"/>
-      <c r="AN27" s="131" t="n"/>
+      <c r="AN27" s="78">
+        <f>Q27*$AN$2</f>
+        <v/>
+      </c>
       <c r="AO27" s="131" t="n"/>
       <c r="AP27" s="135">
         <f>SUM(T27,U27,V27,W27,X27,Y27,Z27,AA27,AB27,AC27,AD27,AE27,AF27,AG27,AH27,AJ27,AK27,AL27,AM27,AN27,AO27)</f>
@@ -7422,8 +7452,8 @@
         <v>0</v>
       </c>
       <c r="AM28" s="130" t="n"/>
-      <c r="AN28" s="130">
-        <f>N26*0.0075</f>
+      <c r="AN28" s="36">
+        <f>Q28*$AN$2</f>
         <v/>
       </c>
       <c r="AO28" s="130" t="n">
@@ -7659,8 +7689,8 @@
         <v>0</v>
       </c>
       <c r="AM29" s="130" t="n"/>
-      <c r="AN29" s="130">
-        <f>N6*0.0075</f>
+      <c r="AN29" s="36">
+        <f>Q29*$AN$2</f>
         <v/>
       </c>
       <c r="AO29" s="130" t="n">
@@ -7896,8 +7926,8 @@
         <v>0</v>
       </c>
       <c r="AM30" s="130" t="n"/>
-      <c r="AN30" s="130">
-        <f>N8*0.0075</f>
+      <c r="AN30" s="36">
+        <f>Q30*$AN$2</f>
         <v/>
       </c>
       <c r="AO30" s="130" t="n">
@@ -8135,8 +8165,8 @@
         <v>0</v>
       </c>
       <c r="AM31" s="130" t="n"/>
-      <c r="AN31" s="130">
-        <f>N7*0.0075</f>
+      <c r="AN31" s="36">
+        <f>Q31*$AN$2</f>
         <v/>
       </c>
       <c r="AO31" s="130" t="n">
@@ -8372,8 +8402,8 @@
         <v>0</v>
       </c>
       <c r="AM32" s="130" t="n"/>
-      <c r="AN32" s="130">
-        <f>N4*0.0075</f>
+      <c r="AN32" s="36">
+        <f>Q32*$AN$2</f>
         <v/>
       </c>
       <c r="AO32" s="130" t="n">
@@ -8609,8 +8639,8 @@
         <v>0</v>
       </c>
       <c r="AM33" s="142" t="n"/>
-      <c r="AN33" s="142">
-        <f>N5*0.0075</f>
+      <c r="AN33" s="48">
+        <f>Q33*$AN$2</f>
         <v/>
       </c>
       <c r="AO33" s="142" t="n">
@@ -8846,8 +8876,8 @@
         <v>0</v>
       </c>
       <c r="AM34" s="130" t="n"/>
-      <c r="AN34" s="130">
-        <f>N13*0.0075</f>
+      <c r="AN34" s="36">
+        <f>Q34*$AN$2</f>
         <v/>
       </c>
       <c r="AO34" s="130" t="n">
@@ -9083,8 +9113,8 @@
         <v>0</v>
       </c>
       <c r="AM35" s="130" t="n"/>
-      <c r="AN35" s="130">
-        <f>N18*0.0075</f>
+      <c r="AN35" s="36">
+        <f>Q35*$AN$2</f>
         <v/>
       </c>
       <c r="AO35" s="130" t="n">
@@ -9320,8 +9350,8 @@
         <v>0</v>
       </c>
       <c r="AM36" s="130" t="n"/>
-      <c r="AN36" s="130">
-        <f>N19*0.0075</f>
+      <c r="AN36" s="36">
+        <f>Q36*$AN$2</f>
         <v/>
       </c>
       <c r="AO36" s="130" t="n">
@@ -9557,8 +9587,8 @@
         <v>0</v>
       </c>
       <c r="AM37" s="130" t="n"/>
-      <c r="AN37" s="130">
-        <f>N20*0.0075</f>
+      <c r="AN37" s="36">
+        <f>Q37*$AN$2</f>
         <v/>
       </c>
       <c r="AO37" s="130" t="n">
@@ -9794,8 +9824,8 @@
         <v>0</v>
       </c>
       <c r="AM38" s="130" t="n"/>
-      <c r="AN38" s="130">
-        <f>N21*0.0075</f>
+      <c r="AN38" s="36">
+        <f>Q38*$AN$2</f>
         <v/>
       </c>
       <c r="AO38" s="130" t="n">
@@ -10031,8 +10061,8 @@
         <v>0</v>
       </c>
       <c r="AM39" s="130" t="n"/>
-      <c r="AN39" s="130">
-        <f>N22*0.0075</f>
+      <c r="AN39" s="36">
+        <f>Q39*$AN$2</f>
         <v/>
       </c>
       <c r="AO39" s="130" t="n">
@@ -10268,8 +10298,8 @@
         <v>0</v>
       </c>
       <c r="AM40" s="130" t="n"/>
-      <c r="AN40" s="130">
-        <f>N14*0.0075</f>
+      <c r="AN40" s="36">
+        <f>Q40*$AN$2</f>
         <v/>
       </c>
       <c r="AO40" s="130" t="n">
@@ -10505,8 +10535,8 @@
         <v>0</v>
       </c>
       <c r="AM41" s="130" t="n"/>
-      <c r="AN41" s="130">
-        <f>N15*0.0075</f>
+      <c r="AN41" s="36">
+        <f>Q41*$AN$2</f>
         <v/>
       </c>
       <c r="AO41" s="130" t="n">
@@ -10742,8 +10772,8 @@
         <v>0</v>
       </c>
       <c r="AM42" s="130" t="n"/>
-      <c r="AN42" s="130">
-        <f>N48*0.0075</f>
+      <c r="AN42" s="36">
+        <f>Q42*$AN$2</f>
         <v/>
       </c>
       <c r="AO42" s="130" t="n">
@@ -10979,8 +11009,8 @@
         <v>0</v>
       </c>
       <c r="AM43" s="130" t="n"/>
-      <c r="AN43" s="130">
-        <f>N49*0.0075</f>
+      <c r="AN43" s="36">
+        <f>Q43*$AN$2</f>
         <v/>
       </c>
       <c r="AO43" s="130" t="n">
@@ -11216,8 +11246,8 @@
         <v>0</v>
       </c>
       <c r="AM44" s="130" t="n"/>
-      <c r="AN44" s="130">
-        <f>N50*0.0075</f>
+      <c r="AN44" s="36">
+        <f>Q44*$AN$2</f>
         <v/>
       </c>
       <c r="AO44" s="130" t="n">
@@ -11453,8 +11483,8 @@
         <v>0</v>
       </c>
       <c r="AM45" s="130" t="n"/>
-      <c r="AN45" s="130">
-        <f>N16*0.0075</f>
+      <c r="AN45" s="36">
+        <f>Q45*$AN$2</f>
         <v/>
       </c>
       <c r="AO45" s="130" t="n">
@@ -11690,8 +11720,8 @@
         <v>0</v>
       </c>
       <c r="AM46" s="130" t="n"/>
-      <c r="AN46" s="130">
-        <f>N10*0.0075</f>
+      <c r="AN46" s="36">
+        <f>Q46*$AN$2</f>
         <v/>
       </c>
       <c r="AO46" s="130" t="n">
@@ -11927,8 +11957,8 @@
         <v>0</v>
       </c>
       <c r="AM47" s="130" t="n"/>
-      <c r="AN47" s="130">
-        <f>N9*0.0075</f>
+      <c r="AN47" s="36">
+        <f>Q47*$AN$2</f>
         <v/>
       </c>
       <c r="AO47" s="130" t="n">
@@ -12164,8 +12194,8 @@
         <v>0</v>
       </c>
       <c r="AM48" s="130" t="n"/>
-      <c r="AN48" s="130">
-        <f>N17*0.0075</f>
+      <c r="AN48" s="36">
+        <f>Q48*$AN$2</f>
         <v/>
       </c>
       <c r="AO48" s="130" t="n">
@@ -12401,8 +12431,8 @@
         <v>0</v>
       </c>
       <c r="AM49" s="130" t="n"/>
-      <c r="AN49" s="130">
-        <f>N47*0.0075</f>
+      <c r="AN49" s="36">
+        <f>Q49*$AN$2</f>
         <v/>
       </c>
       <c r="AO49" s="130" t="n">
@@ -12638,8 +12668,8 @@
         <v>0</v>
       </c>
       <c r="AM50" s="130" t="n"/>
-      <c r="AN50" s="130">
-        <f>N42*0.0075</f>
+      <c r="AN50" s="36">
+        <f>Q50*$AN$2</f>
         <v/>
       </c>
       <c r="AO50" s="130" t="n">
@@ -12875,8 +12905,8 @@
         <v>0</v>
       </c>
       <c r="AM51" s="130" t="n"/>
-      <c r="AN51" s="130">
-        <f>N43*0.0075</f>
+      <c r="AN51" s="36">
+        <f>Q51*$AN$2</f>
         <v/>
       </c>
       <c r="AO51" s="130" t="n">
@@ -13112,8 +13142,8 @@
         <v>0</v>
       </c>
       <c r="AM52" s="130" t="n"/>
-      <c r="AN52" s="130">
-        <f>N44*0.0075</f>
+      <c r="AN52" s="36">
+        <f>Q52*$AN$2</f>
         <v/>
       </c>
       <c r="AO52" s="130" t="n">
@@ -13349,8 +13379,8 @@
         <v>0</v>
       </c>
       <c r="AM53" s="130" t="n"/>
-      <c r="AN53" s="130">
-        <f>N45*0.0075</f>
+      <c r="AN53" s="36">
+        <f>Q53*$AN$2</f>
         <v/>
       </c>
       <c r="AO53" s="130" t="n">
@@ -13586,8 +13616,8 @@
         <v>0</v>
       </c>
       <c r="AM54" s="130" t="n"/>
-      <c r="AN54" s="130">
-        <f>N46*0.0075</f>
+      <c r="AN54" s="36">
+        <f>Q54*$AN$2</f>
         <v/>
       </c>
       <c r="AO54" s="130" t="n">
@@ -14099,7 +14129,7 @@
         <v/>
       </c>
       <c r="AN57" s="56">
-        <f>AVERAGE(AL4:AL50)</f>
+        <f>AVERAGE(AN4:AN54)</f>
         <v/>
       </c>
       <c r="AO57" s="57">
@@ -14446,7 +14476,7 @@
         <v/>
       </c>
       <c r="AN59" s="56">
-        <f>SUM(AL4:AL50)</f>
+        <f>SUM(AN4:AN54)</f>
         <v/>
       </c>
       <c r="AO59" s="57">

</xml_diff>